<commit_message>
working on the user allauth screens
</commit_message>
<xml_diff>
--- a/static/data/teams.xlsx
+++ b/static/data/teams.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdd27291add810d8/projects/teambear/static/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9FE6FE89-180F-4927-9E6A-5088009B4D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="20" documentId="8_{9FE6FE89-180F-4927-9E6A-5088009B4D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44D76AC1-E00A-465F-855B-BEE71B095903}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{5A8766E5-E949-4A74-BFD3-B1D40F8C1DCE}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="612" uniqueCount="254">
   <si>
     <t>team</t>
   </si>
@@ -731,6 +731,57 @@
   </si>
   <si>
     <t>Large free standing mascot teddy bear wearing your teams home football kit</t>
+  </si>
+  <si>
+    <t>ajax</t>
+  </si>
+  <si>
+    <t>arsenal</t>
+  </si>
+  <si>
+    <t>celtic</t>
+  </si>
+  <si>
+    <t>chelsea</t>
+  </si>
+  <si>
+    <t>england</t>
+  </si>
+  <si>
+    <t>everton</t>
+  </si>
+  <si>
+    <t>liverpool</t>
+  </si>
+  <si>
+    <t>rangers</t>
+  </si>
+  <si>
+    <t>wales</t>
+  </si>
+  <si>
+    <t>sunderland</t>
+  </si>
+  <si>
+    <t>astonvilla</t>
+  </si>
+  <si>
+    <t>leeds</t>
+  </si>
+  <si>
+    <t>mancity</t>
+  </si>
+  <si>
+    <t>manutd</t>
+  </si>
+  <si>
+    <t>newcastle</t>
+  </si>
+  <si>
+    <t>realmadrid</t>
+  </si>
+  <si>
+    <t>spurs</t>
   </si>
 </sst>
 </file>
@@ -1608,7 +1659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{28FB3B4E-A0AB-45AA-AAC3-C1F11AABC285}">
-  <dimension ref="A1:M98"/>
+  <dimension ref="A1:O98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -1621,7 +1672,7 @@
     <col min="13" max="13" width="21.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
@@ -1662,7 +1713,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>20</v>
       </c>
@@ -1699,8 +1750,11 @@
       <c r="M2">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O2" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1737,8 +1791,11 @@
       <c r="M3">
         <v>4</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -1775,8 +1832,11 @@
       <c r="M4">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O4" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>20</v>
       </c>
@@ -1813,8 +1873,11 @@
       <c r="M5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1851,8 +1914,11 @@
       <c r="M6">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -1889,8 +1955,11 @@
       <c r="M7">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O7" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>20</v>
       </c>
@@ -1927,8 +1996,11 @@
       <c r="M8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O8" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1965,8 +2037,11 @@
       <c r="M9">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O9" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -2003,8 +2078,11 @@
       <c r="M10">
         <v>4</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O10" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>20</v>
       </c>
@@ -2041,8 +2119,11 @@
       <c r="M11">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O11" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -2079,8 +2160,11 @@
       <c r="M12">
         <v>4</v>
       </c>
-    </row>
-    <row r="13" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O12" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -2117,8 +2201,11 @@
       <c r="M13">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O13" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>20</v>
       </c>
@@ -2155,8 +2242,11 @@
       <c r="M14">
         <v>4</v>
       </c>
-    </row>
-    <row r="15" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O14" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -2193,8 +2283,11 @@
       <c r="M15">
         <v>4</v>
       </c>
-    </row>
-    <row r="16" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O15" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>20</v>
       </c>
@@ -2231,8 +2324,11 @@
       <c r="M16">
         <v>4</v>
       </c>
-    </row>
-    <row r="17" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O16" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>20</v>
       </c>
@@ -2269,8 +2365,11 @@
       <c r="M17">
         <v>4</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="O17" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>65</v>
       </c>
@@ -2308,7 +2407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>65</v>
       </c>
@@ -2346,7 +2445,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>65</v>
       </c>
@@ -2384,7 +2483,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>65</v>
       </c>
@@ -2422,7 +2521,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>65</v>
       </c>
@@ -2460,7 +2559,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -2498,7 +2597,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>65</v>
       </c>
@@ -2536,7 +2635,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -2574,7 +2673,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>65</v>
       </c>
@@ -2612,7 +2711,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>65</v>
       </c>
@@ -2650,7 +2749,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>65</v>
       </c>
@@ -2688,7 +2787,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>65</v>
       </c>
@@ -2726,7 +2825,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>65</v>
       </c>
@@ -2764,7 +2863,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>65</v>
       </c>
@@ -2802,7 +2901,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:15" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>65</v>
       </c>
@@ -2838,6 +2937,9 @@
       </c>
       <c r="M32">
         <v>5</v>
+      </c>
+      <c r="O32" t="s">
+        <v>246</v>
       </c>
     </row>
     <row r="33" spans="1:13" ht="16.5" x14ac:dyDescent="0.25">

</xml_diff>